<commit_message>
add local name and password
</commit_message>
<xml_diff>
--- a/jamin_record.xlsx
+++ b/jamin_record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Appinventiv\Desktop\jamin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CB381DE-5E4C-489B-9528-6984B0778664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B864B97B-E51C-467C-B350-7AE4C7732AD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -311,9 +311,6 @@
     <t>localName</t>
   </si>
   <si>
-    <t>धोबी वाला</t>
-  </si>
-  <si>
     <t>सेमर वाला उत्तर</t>
   </si>
   <si>
@@ -332,9 +329,6 @@
     <t>नगेशेर वाला</t>
   </si>
   <si>
-    <t>चाभ बस</t>
-  </si>
-  <si>
     <t>घर बगीचा</t>
   </si>
   <si>
@@ -378,6 +372,12 @@
   </si>
   <si>
     <t>9817 ,9810 ,9811 , 9810</t>
+  </si>
+  <si>
+    <t>धोबी वाला के बगल में</t>
+  </si>
+  <si>
+    <t>चाभ बास</t>
   </si>
 </sst>
 </file>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1" t="s">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="H2" s="1"/>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H3" s="1"/>
     </row>
@@ -1240,7 +1240,7 @@
         <v>87</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1263,7 +1263,7 @@
         <v>82</v>
       </c>
       <c r="G5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="8" t="s">
-        <v>97</v>
+        <v>112</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="8" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="F8" s="1"/>
       <c r="G8" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1349,7 +1349,7 @@
         <v>88</v>
       </c>
       <c r="G9" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1370,7 +1370,7 @@
       </c>
       <c r="F10" s="1"/>
       <c r="G10" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1391,7 +1391,7 @@
       </c>
       <c r="F11" s="1"/>
       <c r="G11" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1412,7 +1412,7 @@
       </c>
       <c r="F12" s="1"/>
       <c r="G12" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="F14" s="1"/>
       <c r="G14" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="F15" s="1"/>
       <c r="G15" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1496,7 +1496,7 @@
       </c>
       <c r="F16" s="1"/>
       <c r="G16" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="F17" s="1"/>
       <c r="G17" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1540,7 +1540,7 @@
         <v>83</v>
       </c>
       <c r="G18" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="F19" s="1"/>
       <c r="G19" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1569,7 +1569,7 @@
         <v>1450</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>5</v>
@@ -1582,7 +1582,7 @@
       </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="12.5" x14ac:dyDescent="0.25">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="F21" s="1"/>
       <c r="G21" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="12.5" x14ac:dyDescent="0.25">
@@ -1623,7 +1623,7 @@
         <v>84</v>
       </c>
       <c r="G22" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="12.5" x14ac:dyDescent="0.25">
@@ -1631,7 +1631,7 @@
         <v>0</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>46</v>
@@ -1644,7 +1644,7 @@
       </c>
       <c r="F23" s="1"/>
       <c r="G23" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ui and m.k.khan done
</commit_message>
<xml_diff>
--- a/jamin_record.xlsx
+++ b/jamin_record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Appinventiv\Desktop\jamin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B864B97B-E51C-467C-B350-7AE4C7732AD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ECC2BD4-BD6D-4BC7-B824-0F8BEC818C7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -101,9 +101,6 @@
     <t>0.8.6</t>
   </si>
   <si>
-    <t>0.11.13</t>
-  </si>
-  <si>
     <t>0.1.2</t>
   </si>
   <si>
@@ -287,9 +284,6 @@
     <t>9597/12405</t>
   </si>
   <si>
-    <t>wrong correct rakba is 0.5.5</t>
-  </si>
-  <si>
     <t xml:space="preserve">correct will be 0.1.0 </t>
   </si>
   <si>
@@ -378,6 +372,12 @@
   </si>
   <si>
     <t>चाभ बास</t>
+  </si>
+  <si>
+    <t>0.5.5</t>
+  </si>
+  <si>
+    <t>wrong in the list that is 0.11.13</t>
   </si>
 </sst>
 </file>
@@ -755,7 +755,7 @@
     </row>
     <row r="8" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B8" s="1">
         <f t="shared" si="0"/>
@@ -764,7 +764,7 @@
     </row>
     <row r="9" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B9" s="1">
         <f t="shared" si="0"/>
@@ -773,7 +773,7 @@
     </row>
     <row r="10" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B10" s="1">
         <f t="shared" si="0"/>
@@ -782,7 +782,7 @@
     </row>
     <row r="11" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B11" s="1">
         <f t="shared" si="0"/>
@@ -791,7 +791,7 @@
     </row>
     <row r="12" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B12" s="1">
         <f t="shared" si="0"/>
@@ -800,7 +800,7 @@
     </row>
     <row r="13" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B13" s="1">
         <f t="shared" si="0"/>
@@ -809,7 +809,7 @@
     </row>
     <row r="14" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B14" s="1">
         <f t="shared" si="0"/>
@@ -818,7 +818,7 @@
     </row>
     <row r="15" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B15" s="1">
         <f t="shared" si="0"/>
@@ -827,7 +827,7 @@
     </row>
     <row r="16" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B16" s="1">
         <f t="shared" si="0"/>
@@ -836,7 +836,7 @@
     </row>
     <row r="17" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B17" s="1">
         <f t="shared" si="0"/>
@@ -845,7 +845,7 @@
     </row>
     <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B18" s="1">
         <f t="shared" si="0"/>
@@ -854,7 +854,7 @@
     </row>
     <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B19" s="1">
         <f t="shared" si="0"/>
@@ -863,7 +863,7 @@
     </row>
     <row r="20" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B20" s="1">
         <f t="shared" si="0"/>
@@ -872,7 +872,7 @@
     </row>
     <row r="21" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B21" s="1">
         <f t="shared" si="0"/>
@@ -881,7 +881,7 @@
     </row>
     <row r="22" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B22" s="1">
         <f t="shared" si="0"/>
@@ -890,7 +890,7 @@
     </row>
     <row r="23" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B23" s="1">
         <f t="shared" si="0"/>
@@ -899,7 +899,7 @@
     </row>
     <row r="24" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B24" s="1">
         <f t="shared" si="0"/>
@@ -908,7 +908,7 @@
     </row>
     <row r="25" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B25" s="1">
         <f t="shared" si="0"/>
@@ -917,7 +917,7 @@
     </row>
     <row r="26" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B26" s="1">
         <f t="shared" si="0"/>
@@ -998,7 +998,7 @@
     </row>
     <row r="6" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B6" s="1">
         <f t="shared" si="0"/>
@@ -1007,7 +1007,7 @@
     </row>
     <row r="7" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B7" s="1">
         <f t="shared" si="0"/>
@@ -1016,7 +1016,7 @@
     </row>
     <row r="8" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B8" s="1">
         <f t="shared" si="0"/>
@@ -1034,7 +1034,7 @@
     </row>
     <row r="10" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B10" s="1">
         <f t="shared" si="0"/>
@@ -1043,7 +1043,7 @@
     </row>
     <row r="11" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B11" s="1">
         <f t="shared" si="0"/>
@@ -1052,7 +1052,7 @@
     </row>
     <row r="12" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B12" s="1">
         <f t="shared" si="0"/>
@@ -1061,7 +1061,7 @@
     </row>
     <row r="13" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B13" s="1">
         <f t="shared" si="0"/>
@@ -1070,7 +1070,7 @@
     </row>
     <row r="14" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B14" s="1">
         <f t="shared" si="0"/>
@@ -1079,7 +1079,7 @@
     </row>
     <row r="15" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B15" s="1">
         <f t="shared" si="0"/>
@@ -1088,7 +1088,7 @@
     </row>
     <row r="16" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B16" s="1">
         <f t="shared" si="0"/>
@@ -1097,7 +1097,7 @@
     </row>
     <row r="17" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B17" s="1">
         <f t="shared" si="0"/>
@@ -1106,7 +1106,7 @@
     </row>
     <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B18" s="1">
         <f t="shared" si="0"/>
@@ -1115,7 +1115,7 @@
     </row>
     <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B19" s="1">
         <f t="shared" si="0"/>
@@ -1124,7 +1124,7 @@
     </row>
     <row r="20" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B20" s="1">
         <f t="shared" si="0"/>
@@ -1155,25 +1155,25 @@
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>80</v>
-      </c>
       <c r="G1" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1190,11 +1190,11 @@
         <v>37</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H2" s="1"/>
     </row>
@@ -1212,11 +1212,11 @@
         <v>64</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="H3" s="1"/>
     </row>
@@ -1234,13 +1234,13 @@
         <v>25</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1251,19 +1251,19 @@
         <v>9628</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>20</v>
+        <v>111</v>
       </c>
       <c r="D5" s="6">
         <v>87</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>82</v>
+        <v>112</v>
       </c>
       <c r="G5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1274,17 +1274,17 @@
         <v>9615</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D6" s="6">
         <v>56</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1295,17 +1295,17 @@
         <v>9823</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D7" s="6">
         <v>46.2</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="8" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1316,17 +1316,17 @@
         <v>9830</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D8" s="6">
         <v>12</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1337,19 +1337,19 @@
         <v>9834</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D9" s="6">
         <v>30</v>
       </c>
       <c r="E9" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="F9" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="F9" s="8" t="s">
-        <v>88</v>
-      </c>
       <c r="G9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1360,17 +1360,17 @@
         <v>9835</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D10" s="6">
         <v>18</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F10" s="1"/>
       <c r="G10" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1381,17 +1381,17 @@
         <v>9825</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D11" s="6">
         <v>30</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F11" s="1"/>
       <c r="G11" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1402,17 +1402,17 @@
         <v>9826</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D12" s="6">
         <v>29.25</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F12" s="1"/>
       <c r="G12" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1420,7 +1420,7 @@
         <v>1452</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>19</v>
@@ -1429,11 +1429,11 @@
         <v>62</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1444,17 +1444,17 @@
         <v>9759</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D14" s="6">
         <v>23.5</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F14" s="1"/>
       <c r="G14" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1465,17 +1465,17 @@
         <v>9772</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D15" s="6">
         <v>59</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F15" s="1"/>
       <c r="G15" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1486,17 +1486,17 @@
         <v>9781</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D16" s="6">
         <v>27</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F16" s="1"/>
       <c r="G16" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1507,17 +1507,17 @@
         <v>9780</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D17" s="6">
         <v>20.100000000000001</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F17" s="1"/>
       <c r="G17" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1528,19 +1528,19 @@
         <v>9766</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D18" s="6">
         <v>26</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G18" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1551,17 +1551,17 @@
         <v>9614</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D19" s="6">
         <v>24</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F19" s="1"/>
       <c r="G19" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1569,7 +1569,7 @@
         <v>1450</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>5</v>
@@ -1578,11 +1578,11 @@
         <v>26</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="12.5" x14ac:dyDescent="0.25">
@@ -1593,17 +1593,17 @@
         <v>9746</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D21" s="6">
         <v>30</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F21" s="1"/>
       <c r="G21" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="12.5" x14ac:dyDescent="0.25">
@@ -1614,16 +1614,16 @@
         <v>9578</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D22" s="6">
         <v>34.75</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G22" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="12.5" x14ac:dyDescent="0.25">
@@ -1631,20 +1631,20 @@
         <v>0</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D23" s="7">
         <v>0</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F23" s="1"/>
       <c r="G23" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -1744,7 +1744,7 @@
     </row>
     <row r="8" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B8" s="1">
         <f t="shared" si="0"/>
@@ -1762,7 +1762,7 @@
     </row>
     <row r="10" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B10" s="1">
         <f t="shared" si="0"/>
@@ -1771,7 +1771,7 @@
     </row>
     <row r="11" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B11" s="1">
         <f t="shared" si="0"/>
@@ -1780,7 +1780,7 @@
     </row>
     <row r="12" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B12" s="1">
         <f t="shared" si="0"/>
@@ -1789,7 +1789,7 @@
     </row>
     <row r="13" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B13" s="1">
         <f t="shared" si="0"/>
@@ -1798,7 +1798,7 @@
     </row>
     <row r="14" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B14" s="1">
         <f t="shared" si="0"/>
@@ -1807,7 +1807,7 @@
     </row>
     <row r="15" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B15" s="1">
         <f t="shared" si="0"/>
@@ -1816,7 +1816,7 @@
     </row>
     <row r="16" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B16" s="1">
         <f t="shared" si="0"/>
@@ -1825,7 +1825,7 @@
     </row>
     <row r="17" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B17" s="1">
         <f t="shared" si="0"/>
@@ -1834,7 +1834,7 @@
     </row>
     <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B18" s="1">
         <f t="shared" si="0"/>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B19" s="1">
         <f t="shared" si="0"/>
@@ -1861,7 +1861,7 @@
     </row>
     <row r="21" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B21" s="1">
         <f t="shared" si="0"/>
@@ -1870,7 +1870,7 @@
     </row>
     <row r="22" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B22" s="1">
         <f t="shared" si="0"/>
@@ -1879,7 +1879,7 @@
     </row>
     <row r="23" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B23" s="1">
         <f t="shared" si="0"/>
@@ -1888,7 +1888,7 @@
     </row>
     <row r="24" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B24" s="1">
         <f t="shared" si="0"/>
@@ -1910,7 +1910,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B1" s="1">
         <f t="shared" ref="B1:B20" si="0">LEFT(A1,FIND(".",A1)-1)*400 + MID(A1,FIND(".",A1)+1,FIND(".",A1,FIND(".",A1)+1)-FIND(".",A1)-1)*20 + RIGHT(A1,LEN(A1)-FIND(".",A1,FIND(".",A1)+1))</f>
@@ -1927,7 +1927,7 @@
     </row>
     <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B2" s="1">
         <f t="shared" si="0"/>
@@ -1942,7 +1942,7 @@
     </row>
     <row r="3" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B3" s="1">
         <f t="shared" si="0"/>
@@ -1951,7 +1951,7 @@
     </row>
     <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B4" s="1">
         <f t="shared" si="0"/>
@@ -1969,7 +1969,7 @@
     </row>
     <row r="6" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B6" s="1">
         <f t="shared" si="0"/>
@@ -1987,7 +1987,7 @@
     </row>
     <row r="8" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B8" s="1">
         <f t="shared" si="0"/>
@@ -1996,7 +1996,7 @@
     </row>
     <row r="9" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B9" s="1">
         <f t="shared" si="0"/>
@@ -2005,7 +2005,7 @@
     </row>
     <row r="10" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B10" s="1">
         <f t="shared" si="0"/>
@@ -2014,7 +2014,7 @@
     </row>
     <row r="11" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B11" s="1">
         <f t="shared" si="0"/>
@@ -2023,7 +2023,7 @@
     </row>
     <row r="12" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B12" s="1">
         <f t="shared" si="0"/>
@@ -2032,7 +2032,7 @@
     </row>
     <row r="13" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B13" s="1">
         <f t="shared" si="0"/>
@@ -2041,7 +2041,7 @@
     </row>
     <row r="14" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B14" s="1">
         <f t="shared" si="0"/>
@@ -2050,7 +2050,7 @@
     </row>
     <row r="15" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B15" s="1">
         <f t="shared" si="0"/>
@@ -2059,7 +2059,7 @@
     </row>
     <row r="16" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B16" s="1">
         <f t="shared" si="0"/>
@@ -2068,7 +2068,7 @@
     </row>
     <row r="17" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B17" s="1">
         <f t="shared" si="0"/>
@@ -2077,7 +2077,7 @@
     </row>
     <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B18" s="1">
         <f t="shared" si="0"/>
@@ -2086,7 +2086,7 @@
     </row>
     <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B19" s="1">
         <f t="shared" si="0"/>
@@ -2117,7 +2117,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B1" s="1">
         <f>LEFT(A1,FIND(".",A1)-1)*400 + MID(A1,FIND(".",A1)+1,FIND(".",A1,FIND(".",A1)+1)-FIND(".",A1)-1)*20 + RIGHT(A1,LEN(A1)-FIND(".",A1,FIND(".",A1)+1))</f>

</xml_diff>